<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-04 Sarah souffle et fait une pause
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-04.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'étoile de pâte de Mila</t>
+          <t>Sarah souffle et fait une pause</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine</t>
+          <t>cuisine, table, pâte, rouleau, bois, fenêtre, rayon, beurre, moule, formes</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, papa, maman</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut coller des formes en pâte. Une forme se casse. Elle souffle, fait une pause, puis pose une étoile.</t>
+          <t>Le bois du rouleau luit près de la fenêtre. Près du bois, un éclat de rouleau brille. Sarah veut coller, maintenant. Forme cassée, poitrine trop vite, sourire parti, papa accroupi. Elle souffle, pause. Merci vécu. 2e ruse : le cœur se plie sous le rouleau. Un éclat de rouleau tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cuisine, un rayon traverse la farine. La farine danse, toute légère. Des grains blancs tournent dans la lumière. La cuillère en bois tape le saladier. Ça sent le beurre. Ça sent aussi le lait tiède. La pâte est prête, Mila. Je pose un bol près de la plaque. Tes mains vont dans la farine. Tout doux. Elle est froide, la pâte. Oui. Un peu froide. Ça sent bon. On va coller des formes, ensemble. En ce moment, Mila est à table. Elle colle des formes en pâte. Un rond. Un cœur. Une étoile. Tu appuies sans presser trop ? Oui. Une belle étoile. Mila appuie le moule. La pâte se déchire. La forme se casse. Mila sent sa poitrine aller vite. Ses joues chauffent. C'est trop. Je suis fâchée. La forme s'est cassée. Tu es fâchée. On peut souffler. On peut faire une pause. Mila s'assoit bien sur sa chaise. Elle pose les mains sur ses genoux. Elle souffle comme le vent. Une fois. Deux fois. Elle fait une pause. La cuisine redevient calme. La farine retombe, toute fine. Je souffle. Je fais une pause. Bravo. Ton corps ralentit. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Un nouveau morceau. Mila reprend un morceau de pâte. Elle l'étale tout doucement. La pâte sent encore la farine.</t>
+          <t>Le bois du rouleau luit près de la fenêtre. Ça sent le beurre, un peu. Ça sent bon, papa. Tu le sens, le beurre, Sarah ? Oui, papa. Un rayon glisse sur le bois. Il brille, maman. Le rouleau est lisse ? Un peu, maman. La pâte attend sur la table. On colle des formes, d'accord ? Oui, papa. Un fil de pâte pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La pâte est froide contre la peau. Elle colle, maman. Tu la sens, la pâte ? Oui. Près du bois, un éclat de rouleau brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du bois. Elle vole, maman. Au-dessus du rouleau ? Oui, au-dessus. Papa pose le moule près de la pâte. Le moule est un peu lourd. On colle l'étoile, papa ? Le saladier tape le bois. La pâte s'étale un peu. C'est blanc, papa. Comme un nuage ? Oui, comme un nuage. En ce moment, Sarah appuie le moule sur la pâte. Je veux coller, maintenant ! L'étoile, tout de suite. Tu vois le moule, Sarah ? Oui, papa. Sarah appuie trop fort. La pâte se déchire. La forme se casse. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle casse, Sarah ? Oui, papa. Tes lèvres sont serrées, Sarah ? Un peu, maman. L'éclat de rouleau tremble, puis tient. Sarah serre le moule contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cuisine, un rayon traverse la farine. La farine danse, toute légère. Des grains blancs tournent dans la lumière. La cuillère en bois tape le saladier. Ça sent le beurre. Ça sent aussi le lait tiède. La pâte est prête, Mila. Je pose un bol près de la plaque. Tes mains vont dans la farine. Tout doux. Elle est froide, la pâte. Oui. Un peu froide. Ça sent bon. On va coller des formes, ensemble. En ce moment, Mila est à table. Elle colle des formes en pâte. Un rond. Un cœur. Une étoile. Tu appuies sans presser trop ? Oui. Une belle étoile. Mila appuie le moule. La pâte se déchire. La forme se casse. Mila sent sa poitrine aller vite. Ses joues chauffent. C'est trop. Je suis fâchée. La forme s'est cassée. Tu es fâchée. On peut souffler. On peut faire une pause. Mila s'assoit bien sur sa chaise. Elle pose les mains sur ses genoux. Elle souffle comme le vent. Une fois. Deux fois. Elle fait une pause. La cuisine redevient calme. La farine retombe, toute fine. Je souffle. Je fais une pause. Bravo. Ton corps ralentit. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Un nouveau morceau. Mila reprend un morceau de pâte. Elle l'étale tout doucement. La pâte sent encore la farine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois du rouleau luit près de la fenêtre. Ça sent le beurre, un peu. Ça sent bon, papa. Tu le sens, le beurre, Sarah ? Oui, papa. Un rayon glisse sur le bois. Il brille, maman. Le rouleau est lisse ? Un peu, maman. La pâte attend sur la table. On colle des formes, d'accord ? Oui, papa. Un fil de pâte pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La pâte est froide contre la peau. Elle colle, maman. Tu la sens, la pâte ? Oui. Près du bois, un &lt;emphasis level="moderate"&gt;éclat de rouleau&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du bois. Elle vole, maman. Au-dessus du rouleau ? Oui, au-dessus. Papa pose le moule près de la pâte. Le moule est un peu lourd. On colle l'étoile, papa ? Le saladier tape le bois. La pâte s'étale un peu. C'est blanc, papa. Comme un nuage ? Oui, comme un nuage. En ce moment, Sarah appuie le moule sur la pâte. Je veux coller, maintenant ! L'étoile, tout de suite. Tu vois le moule, Sarah ? Oui, papa. Sarah appuie trop fort. La pâte se déchire. La forme se casse. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle casse, Sarah ? Oui, papa. Tes lèvres sont serrées, Sarah ? Un peu, maman. L'éclat de rouleau tremble, puis tient. Sarah serre le moule contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Paloma est dans la cuisine avec papa. Ils collent des formes en pâte. La pâte est froide. Une forme se casse. Paloma sent sa poitrine aller vite. Ses joues chauffent. Elle dit : c'est trop. Papa est là, près de la table. Papa dit : on peut &lt;emphasis&gt;souffler&lt;/emphasis&gt;. Paloma souffle comme le vent. Une fois. Deux fois. Elle s'assoit. Elle fait une pause. Ses mains se posent sur ses genoux. La cuisine redevient calme. Parce qu'elle a soufflé, son corps ralentit. Paloma reprend un morceau de pâte. Elle l'étale tout doucement. Papa reste près d'elle. Plus tard, une autre forme se plie. Paloma sent encore la poitrine vite. Elle souffle. Elle fait une pause. Elle s'assoit. Puis elle reprend. Papa dit : souffler, puis une pause. On peut reprendre. Paloma pose une étoile. La pâte sent la farine. [pause]</t>
+          <t>Le bois du rouleau luit près de la fenêtre. Ça sent le beurre, un peu. Ça sent bon, papa. Tu le sens, le beurre, Sarah ? Oui, papa. Un rayon glisse sur le bois. Il brille, maman. Le rouleau est lisse ? Un peu, maman. La pâte attend sur la table. On colle des formes, d'accord ? Oui, papa. Un fil de pâte pend vers le bois. Il pend, papa. Tu le vois, le fil ? Oui. La pâte est froide contre la peau. Elle colle, maman. Tu la sens, la pâte ? Oui. Près du bois, un &lt;emphasis&gt;éclat de rouleau&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du bois. Elle vole, maman. Au-dessus du rouleau ? Oui, au-dessus. Papa pose le moule près de la pâte. Le moule est un peu lourd. On colle l'étoile, papa ? Le saladier tape le bois. La pâte s'étale un peu. C'est blanc, papa. Comme un nuage ? Oui, comme un nuage. En ce moment, Sarah appuie le moule sur la pâte. Je veux coller, maintenant ! L'étoile, tout de suite. Tu vois le moule, Sarah ? Oui, papa. Sarah appuie trop fort. La pâte se déchire. La forme se casse. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules montent un peu. Elle casse, Sarah ? Oui, papa. Tes lèvres sont serrées, Sarah ? Un peu, maman. L'éclat de rouleau tremble, puis tient. Sarah serre le moule contre elle. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat de rouleau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,51 +1321,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=elle_veut_coller_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dans la cuisine, un rayon traverse la farine.
-narrateur|La farine danse, toute légère.
-narrateur|Des grains blancs tournent dans la lumière.
-narrateur|La cuillère en bois tape le saladier.
-narrateur|Ça sent le beurre.
-narrateur|Ça sent aussi le lait tiède.
-papa|La pâte est prête, Mila.
-maman|Je pose un bol près de la plaque.
-papa|Tes mains vont dans la farine. Tout doux.
-enfant-f|Elle est froide, la pâte.
-maman|Oui. Un peu froide. Ça sent bon.
-papa|On va coller des formes, ensemble.
-narrateur|En ce moment, Mila est à table.
-narrateur|Elle colle des formes en pâte.
-narrateur|Un rond. Un cœur. Une étoile.
-papa|Tu appuies sans presser trop ?
-enfant-f|Oui. Une belle étoile.
-narrateur|Mila appuie le moule.
+          <t>narrateur|Le bois du rouleau luit près de la fenêtre.
+narrateur|Ça sent le beurre, un peu.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le beurre, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Un rayon glisse sur le bois.
+enfant-f|Il brille, maman.
+maman|Le rouleau est lisse ?
+enfant-f|Un peu, maman.
+maman|La pâte attend sur la table.
+papa|On colle des formes, d'accord ?
+enfant-f|Oui, papa.
+narrateur|Un fil de pâte pend vers le bois.
+enfant-f|Il pend, papa.
+papa|Tu le vois, le fil ?
+enfant-f|Oui.
+narrateur|La pâte est froide contre la peau.
+enfant-f|Elle colle, maman.
+maman|Tu la sens, la pâte ?
+enfant-f|Oui.
+narrateur|Près du bois, un éclat de rouleau brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Une poussière danse au-dessus du bois.
+enfant-f|Elle vole, maman.
+maman|Au-dessus du rouleau ?
+enfant-f|Oui, au-dessus.
+narrateur|Papa pose le moule près de la pâte.
+narrateur|Le moule est un peu lourd.
+enfant-f|On colle l'étoile, papa ?
+narrateur|Le saladier tape le bois.
+narrateur|La pâte s'étale un peu.
+enfant-f|C'est blanc, papa.
+papa|Comme un nuage ?
+enfant-f|Oui, comme un nuage.
+narrateur|En ce moment, Sarah appuie le moule sur la pâte.
+enfant-f|Je veux coller, maintenant !
+enfant-f|L'étoile, tout de suite.
+papa|Tu vois le moule, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Sarah appuie trop fort.
 narrateur|La pâte se déchire.
 narrateur|La forme se casse.
-narrateur|Mila sent sa poitrine aller vite.
-narrateur|Ses joues chauffent.
-enfant-f|C'est trop. Je suis fâchée.
-papa|La forme s'est cassée. Tu es fâchée.
-papa|On peut souffler.
-maman|On peut faire une pause.
-narrateur|Mila s'assoit bien sur sa chaise.
-narrateur|Elle pose les mains sur ses genoux.
-narrateur|Elle souffle comme le vent.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Elle fait une pause.
-narrateur|La cuisine redevient calme.
-narrateur|La farine retombe, toute fine.
-enfant-f|Je souffle. Je fais une pause.
-maman|Bravo. Ton corps ralentit.
-papa|Tu as soufflé. Tu as fait une pause.
-papa|Tu veux reprendre, tout doucement ?
-enfant-f|Oui. Un nouveau morceau.
-narrateur|Mila reprend un morceau de pâte.
-narrateur|Elle l'étale tout doucement.
-narrateur|La pâte sent encore la farine.</t>
+enfant-f|Oh.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules montent un peu.
+papa|Elle casse, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont serrées, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de rouleau tremble, puis tient.
+narrateur|Sarah serre le moule contre elle.
+enfant-f|C'est trop, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Sarah regarde papa.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1397,17 +1416,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Mila va vite. Que fait-elle ?</t>
+          <t>Le corps de Sarah va vite. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Mila va vite. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps de &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; va vite. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le corps de Paloma va vite. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps de &lt;emphasis&gt;Sarah&lt;/emphasis&gt; va vite. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1432,7 +1451,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Papa dit de souffler. Que fait Paloma ensuite ?</t>
+          <t>Papa dit de souffler. Que fait Sarah ensuite ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1470,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1481,7 +1500,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1496,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1538,22 +1561,22 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_corps_de_sarah_va_vite_que_fait_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le corps de Mila va vite.
+          <t>narrateur|Le corps de Sarah va vite.
 narrateur|Que fait-elle ?</t>
         </is>
       </c>
@@ -1581,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a soufflé. Elle a fait une pause. Son corps a ralenti. La farine sent encore le blé. Ça sent le beurre aussi. Oui. On reste à table, ensemble. Plus tard, une autre forme se plie. Mila sent encore la poitrine vite. Je souffle. Je fais une pause. Oui. Souffler, puis une pause. On peut reprendre. Mila s'assoit. Elle souffle. Elle fait une pause. Tes mains sont sur tes genoux. C'est bien. Mila reprend la pâte. Elle l'étale, tout plat. Elle pose une étoile. L'étoile est entière. Bravo.</t>
+          <t>Sarah veut coller, tout de suite. Je colle, maintenant ! Elle appuie trop vite sur la pâte. Le moule déchire la forme. Sarah baisse les yeux. Sa poitrine est coincée. C'est trop. Sarah souffle, un filet d'air. Une fois. Deux fois. Elle fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le rouleau, un instant. Elle écoute le silence de la cuisine. Tu veux coller l'étoile ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle, plus loin. La pâte s'arrête de bouger. L'étoile. J'aime l'étoile. Maman pose le moule sur la table. Merci, Sarah. Papa reste près du bois. La pâte est tiède, sous les doigts. Elle est froide. La forme tient, un peu de travers. L'étoile. Elle a cinq branches, là ? Oui, là. Sarah glisse la main près du rouleau. Le bois est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Sarah s'assoit, puis se relève. On la pose au bord ? La pâte va jusqu'à la plaque. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a soufflé. Elle a fait une pause. Son corps a ralenti. La farine sent encore le blé. Ça sent le beurre aussi. Oui. On reste à table, ensemble. Plus tard, une autre forme se plie. Mila sent encore la poitrine vite. Je souffle. Je fais une pause. Oui. Souffler, puis une pause. On peut reprendre. Mila s'assoit. Elle souffle. Elle fait une pause. Tes mains sont sur tes genoux. C'est bien. Mila reprend la pâte. Elle l'étale, tout plat. Elle pose une étoile. L'étoile est entière. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut coller, tout de suite. Je colle, maintenant ! Elle appuie trop vite sur la pâte. Le moule déchire la forme. Sarah baisse les yeux. Sa poitrine est coincée. C'est trop. Sarah &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt;, un filet d'air. Une fois. Deux fois. Elle fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le rouleau, un instant. Elle écoute le silence de la cuisine. Tu veux coller l'étoile ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle, plus loin. La pâte s'arrête de bouger. L'étoile. J'aime l'étoile. Maman pose le moule sur la table. Merci, Sarah. Papa reste près du bois. La pâte est tiède, sous les doigts. Elle est froide. La forme tient, un peu de travers. L'étoile. Elle a cinq branches, là ? Oui, là. Sarah glisse la main près du rouleau. Le bois est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Sarah s'assoit, puis se relève. On la pose au bord ? La pâte va jusqu'à la plaque. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Paloma a soufflé. Elle a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Son corps a ralenti. [pause]</t>
+          <t>Sarah veut coller, tout de suite. Je colle, maintenant ! Elle appuie trop vite sur la pâte. Le moule déchire la forme. Sarah baisse les yeux. Sa poitrine est coincée. C'est trop. Sarah &lt;emphasis&gt;souffle&lt;/emphasis&gt;, un filet d'air. Une fois. Deux fois. Elle fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Elle observe le rouleau, un instant. Elle écoute le silence de la cuisine. Tu veux coller l'étoile ? Papa reste à la même hauteur. Papa, on fait quoi ? On laisse un peu d'air ? D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle, plus loin. La pâte s'arrête de bouger. L'étoile. J'aime l'étoile. Maman pose le moule sur la table. Merci, Sarah. Papa reste près du bois. La pâte est tiède, sous les doigts. Elle est froide. La forme tient, un peu de travers. L'étoile. Elle a cinq branches, là ? Oui, là. Sarah glisse la main près du rouleau. Le bois est lisse, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Sarah s'assoit, puis se relève. On la pose au bord ? La pâte va jusqu'à la plaque. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1638,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1646,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1672,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,29 +1743,53 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=gêne puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_souffle_elle_fait_une_pause; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a soufflé.
-narrateur|Elle a fait une pause.
-narrateur|Son corps a ralenti.
-maman|La farine sent encore le blé.
-enfant-f|Ça sent le beurre aussi.
-papa|Oui. On reste à table, ensemble.
-narrateur|Plus tard, une autre forme se plie.
-narrateur|Mila sent encore la poitrine vite.
-enfant-f|Je souffle. Je fais une pause.
-papa|Oui. Souffler, puis une pause. On peut reprendre.
-narrateur|Mila s'assoit.
-narrateur|Elle souffle.
+          <t>narrateur|Sarah veut coller, tout de suite.
+enfant-f|Je colle, maintenant !
+narrateur|Elle appuie trop vite sur la pâte.
+narrateur|Le moule déchire la forme.
+narrateur|Sarah baisse les yeux.
+narrateur|Sa poitrine est coincée.
+enfant-f|C'est trop.
+narrateur|Sarah souffle, un filet d'air.
+narrateur|Une fois.
+narrateur|Deux fois.
 narrateur|Elle fait une pause.
-maman|Tes mains sont sur tes genoux. C'est bien.
-narrateur|Mila reprend la pâte.
-narrateur|Elle l'étale, tout plat.
-narrateur|Elle pose une étoile.
-papa|L'étoile est entière. Bravo.</t>
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne parle.
+narrateur|Elle observe le rouleau, un instant.
+narrateur|Elle écoute le silence de la cuisine.
+papa|Tu veux coller l'étoile ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On laisse un peu d'air ?
+enfant-f|D'accord.
+narrateur|Sarah reste un moment, les mains ouvertes.
+narrateur|Elle souffle, plus loin.
+narrateur|La pâte s'arrête de bouger.
+enfant-f|L'étoile.
+enfant-f|J'aime l'étoile.
+narrateur|Maman pose le moule sur la table.
+papa|Merci, Sarah.
+narrateur|Papa reste près du bois.
+maman|La pâte est tiède, sous les doigts.
+enfant-f|Elle est froide.
+narrateur|La forme tient, un peu de travers.
+enfant-f|L'étoile.
+papa|Elle a cinq branches, là ?
+enfant-f|Oui, là.
+narrateur|Sarah glisse la main près du rouleau.
+narrateur|Le bois est lisse, contre la peau.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Sarah s'assoit, puis se relève.
+enfant-f|On la pose au bord ?
+maman|La pâte va jusqu'à la plaque.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1774,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila porte l'étoile jusqu'à la plaque. La plaque est froide et lisse. Elle va cuire, maman ? Oui. Papa met la plaque. Tu as fini ta forme ? Oui. J'ai soufflé aussi. Mila essuie un peu de farine. La cuisine sent encore le beurre. On lave les mains ensemble ? Oui. Après l'étoile.</t>
+          <t>Ils restent près de la table. La pâte tombe d'un côté. Le cœur, maintenant ! Sarah appuie le moule trop vite. La forme colle au bois. Elle part ! Le cœur se plie, sous le rouleau. La pâte tire trop fort, cette fois. Oh. Sarah souffle, un filet d'air. Elle fait une pause, sous le rayon. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah souffle, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bois, un instant. Elle écoute le silence de la cuisine. Au bord du bois, un éclat de rouleau luit. Là, sur le rouleau. Tu veux le cœur, maman ? Maman ne presse plus. Elle tend le moule, sans serrer. Je prends le cœur. Sarah étale la pâte, sans se presser. Maman la reçoit, plus loin. La pâte est lisse et froide. Tu le vois, le cœur ? Oui, papa. La forme est près de la plaque ? Oui, maman. Maman pose un bord. Sarah pose une main sur le bois. La forme tient, Sarah ? Oui, papa. Un rayon passe sur le rouleau. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila porte l'étoile jusqu'à la plaque. La plaque est froide et lisse. Elle va cuire, maman ? Oui. Papa met la plaque. Tu as fini ta forme ? Oui. J'ai soufflé aussi. Mila essuie un peu de farine. La cuisine sent encore le beurre. On lave les mains ensemble ? Oui. Après l'étoile.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de la table. La pâte tombe d'un côté. Le cœur, maintenant ! Sarah appuie le moule trop vite. La forme colle au bois. Elle part ! Le cœur se plie, sous le rouleau. La pâte tire trop fort, cette fois. Oh. Sarah souffle, un filet d'air. Elle fait une pause, sous le rayon. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah souffle, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bois, un instant. Elle écoute le silence de la cuisine. Au bord du bois, un &lt;emphasis level="moderate"&gt;éclat de rouleau&lt;/emphasis&gt; luit. Là, sur le rouleau. Tu veux le cœur, maman ? Maman ne presse plus. Elle tend le moule, sans serrer. Je prends le cœur. Sarah étale la pâte, sans se presser. Maman la reçoit, plus loin. La pâte est lisse et froide. Tu le vois, le cœur ? Oui, papa. La forme est près de la plaque ? Oui, maman. Maman pose un bord. Sarah pose une main sur le bois. La forme tient, Sarah ? Oui, papa. Un rayon passe sur le rouleau. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Paloma pose l'étoile sur la plaque. Papa reste à côté. [pause]</t>
+          <t>Ils restent près de la table. La pâte tombe d'un côté. Le cœur, maintenant ! Sarah appuie le moule trop vite. La forme colle au bois. Elle part ! Le cœur se plie, sous le rouleau. La pâte tire trop fort, cette fois. Oh. Sarah souffle, un filet d'air. Elle fait une pause, sous le rayon. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah souffle, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le bois, un instant. Elle écoute le silence de la cuisine. Au bord du bois, un &lt;emphasis&gt;éclat de rouleau&lt;/emphasis&gt; luit. Là, sur le rouleau. Tu veux le cœur, maman ? Maman ne presse plus. Elle tend le moule, sans serrer. Je prends le cœur. Sarah étale la pâte, sans se presser. Maman la reçoit, plus loin. La pâte est lisse et froide. Tu le vois, le cœur ? Oui, papa. La forme est près de la plaque ? Oui, maman. Maman pose un bord. Sarah pose une main sur le bois. La forme tient, Sarah ? Oui, papa. Un rayon passe sur le rouleau. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1831,7 +1878,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1839,10 +1886,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1863,28 +1910,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rouleau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1893,10 +1944,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1907,18 +1958,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=coeur_plie_sous_le_rouleau_elle_souffle; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila porte l'étoile jusqu'à la plaque.
-narrateur|La plaque est froide et lisse.
-enfant-f|Elle va cuire, maman ?
-maman|Oui. Papa met la plaque. Tu as fini ta forme ?
-enfant-f|Oui. J'ai soufflé aussi.
-narrateur|Mila essuie un peu de farine.
-narrateur|La cuisine sent encore le beurre.
-maman|On lave les mains ensemble ?
-enfant-f|Oui. Après l'étoile.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|La pâte tombe d'un côté.
+enfant-f|Le cœur, maintenant !
+narrateur|Sarah appuie le moule trop vite.
+narrateur|La forme colle au bois.
+enfant-f|Elle part !
+narrateur|Le cœur se plie, sous le rouleau.
+narrateur|La pâte tire trop fort, cette fois.
+enfant-f|Oh.
+narrateur|Sarah souffle, un filet d'air.
+narrateur|Elle fait une pause, sous le rayon.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah souffle, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le bois, un instant.
+narrateur|Elle écoute le silence de la cuisine.
+narrateur|Au bord du bois, un éclat de rouleau luit.
+enfant-f|Là, sur le rouleau.
+enfant-f|Tu veux le cœur, maman ?
+narrateur|Maman ne presse plus.
+narrateur|Elle tend le moule, sans serrer.
+maman|Je prends le cœur.
+narrateur|Sarah étale la pâte, sans se presser.
+narrateur|Maman la reçoit, plus loin.
+narrateur|La pâte est lisse et froide.
+papa|Tu le vois, le cœur ?
+enfant-f|Oui, papa.
+maman|La forme est près de la plaque ?
+enfant-f|Oui, maman.
+narrateur|Maman pose un bord.
+narrateur|Sarah pose une main sur le bois.
+papa|La forme tient, Sarah ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le rouleau.
+enfant-f|Il allume le bois.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1950,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Mila. L'étoile est sur la plaque.</t>
+          <t>Ils restent près de la table. L'étoile est arrivée, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. La pâte sent le beurre. Tu le sens, le beurre ? Oui, maman. La forme reste un peu, de travers. Elle a tenu, sur la plaque. La plaque. La pâte est froide, sous les mains. Le rouleau de bois fait de l'ombre. On y retourne, après. Un éclat de rouleau tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Mila. L'étoile est sur la plaque.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. L'étoile est arrivée, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. La pâte sent le beurre. Tu le sens, le beurre ? Oui, maman. La forme reste un peu, de travers. Elle a tenu, sur la plaque. La plaque. La pâte est froide, sous les mains. Le rouleau de bois fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de rouleau&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. L'étoile est arrivée, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. La pâte sent le beurre. Tu le sens, le beurre ? Oui, maman. La forme reste un peu, de travers. Elle a tenu, sur la plaque. La plaque. La pâte est froide, sous les mains. Le rouleau de bois fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de rouleau&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,7 +2090,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2015,10 +2098,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rouleau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,26 +2160,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai soufflé. J'ai fait une pause.
-papa|Bravo, Mila.
-maman|L'étoile est sur la plaque.</t>
+          <t>narrateur|Ils restent près de la table.
+maman|L'étoile est arrivée, Sarah ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle, un filet d'air.
+enfant-f|La pâte sent le beurre.
+maman|Tu le sens, le beurre ?
+enfant-f|Oui, maman.
+papa|La forme reste un peu, de travers.
+enfant-f|Elle a tenu, sur la plaque.
+maman|La plaque.
+narrateur|La pâte est froide, sous les mains.
+narrateur|Le rouleau de bois fait de l'ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat de rouleau tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2177,6 +2281,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>